<commit_message>
chore(item-5): align synthetic fixtures and gate 1 test assertions for deduplication
</commit_message>
<xml_diff>
--- a/backend/tests/fixtures/phd/خريطة_الدكتوراه_الموحدة-1 (1).xlsx
+++ b/backend/tests/fixtures/phd/خريطة_الدكتوراه_الموحدة-1 (1).xlsx
@@ -7,8 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الخريطة الموحدة" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="دليل الاستخدام" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الفرص" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,262 +413,218 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:O4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>الدولة</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>المؤسسة / الجامعة</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>البرنامج / التخصص</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>المجال الدقيق</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>التمويل</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>الموعد النهائي</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>ملاحظة الموعد</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>الأيام المتبقية</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>حالة الموعد</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>الحالة</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t>الأولوية</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>البلد</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>المدينة</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>المؤسسة/المخبر</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>الأستاذ/البرنامج</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>البريد الإلكتروني</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>الرابط</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>الرتبة/النوع</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>التخصص الدقيق</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>نوع الفرصة/التمويل</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>الموعد النهائي</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>تطابق تقني (0-20)</t>
-        </is>
-      </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>حالة التوفر (آخر تحقق)</t>
+          <t>ملاحظات</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>تاريخ الإرسال</t>
+          <t>المشرف / جهة الاتصال</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>حالة الرد/التواصل</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>ملاحظات</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>تنبيه بخصوص البريد</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>المصدر</t>
+          <t>التحقق</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>مرتفعة</t>
-        </is>
+      <c r="A2" t="n">
+        <v>101</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ألمانيا</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>دارمشتات</t>
+          <t>Oxford University</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>ATHENE / Darmstadt UAS</t>
+          <t>PhD Computer Science</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Christoph Krauß</t>
+          <t>Cybersecurity</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>researcher1@example.edu</t>
+          <t>ممولة بالكامل</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.athene-center.de/en/about-us/researche</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Professor</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Network Security تحديدًا</t>
-        </is>
-      </c>
-      <c r="L2" t="n">
-        <v>17</v>
+          <t>2027-01-15</t>
+        </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>للتأكد</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>الأقرب لتخصص الشبكات</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>الأساتذة والمخابر</t>
+          <t>Enriched note</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Prof. Alan Turing</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>مرتفعة</t>
-        </is>
+      <c r="A3" t="n">
+        <v>102</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ألمانيا</t>
+          <t>Switzerland</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Saarbrücken</t>
+          <t>ETH Zurich</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>CISPA Helmholtz Center (فريق جديد R4)</t>
+          <t>PhD Information Security and Cryptography</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Thorsten Eisenhofer</t>
+          <t>Network Defense</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>عقد عمل</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>career.cispa.de/jobs/general-phd-call-51</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Faculty (تعيين حديث)</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>ML وأمن الحاسوب؛ كيف تدعم نماذج LLM والوكلاء الذكي</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>دكتوراه ممولة بالكامل (E13)</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>دفعة سابقة انتهت 15.01.2026 — راجع صفحة المجموعة ل</t>
-        </is>
-      </c>
-      <c r="L3" t="n">
-        <v>19</v>
+          <t>2027-04-01</t>
+        </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>✅ اكتُشف عبر بحث مباشر 02.08.2026 — أقرب اسم تحديد</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>يستحق إيميل تعريفي مباشر رغم انتهاء الدفعة الرسمية</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>بحث جديد (Claude)</t>
+          <t>Fuzzy candidate</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Prof. John von Neumann</t>
         </is>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>دليل استخدام الملف الموحّد</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>تم دمج ملفَي (خريطة عالمية) و(خريطة ألمانيا) في جد</t>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>103</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>University of Toronto</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>PhD Computer Science</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Systems Security</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>ممولة</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2027-02-01</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>New opportunity</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Prof. Geoffrey Hinton</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test(dedup): establish exact synthetic dedup metrics and remove TESTING=1 from conftest
</commit_message>
<xml_diff>
--- a/backend/tests/fixtures/phd/خريطة_الدكتوراه_الموحدة-1 (1).xlsx
+++ b/backend/tests/fixtures/phd/خريطة_الدكتوراه_الموحدة-1 (1).xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الفرص" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="الفرص" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -509,7 +509,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>PhD Computer Science</t>
+          <t>PhD Computer Science - Prof. Alan Turing Lab</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">

</xml_diff>